<commit_message>
add permission on view and web route
</commit_message>
<xml_diff>
--- a/public/download/template_siswa.xlsx
+++ b/public/download/template_siswa.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Applications/MAMP/htdocs/computer-assisted-test/public/download/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6C7F39C-8182-5F4A-9AC8-542A86D433DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F0AC0E33-95CC-9444-8632-7909CF303E77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="38400" windowHeight="20060" xr2:uid="{F2F64410-2DB0-454A-95F9-BACD18C62E9B}"/>
   </bookViews>
@@ -25,10 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
-  <si>
-    <t>No</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
   <si>
     <t>Nama</t>
   </si>
@@ -43,9 +40,6 @@
   </si>
   <si>
     <t>XI-A</t>
-  </si>
-  <si>
-    <t>Username</t>
   </si>
   <si>
     <t>Habib</t>
@@ -421,65 +415,45 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91EE5671-6C78-D744-92D9-A6163445A131}">
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="6" customWidth="1"/>
-    <col min="2" max="2" width="32.1640625" customWidth="1"/>
-    <col min="3" max="3" width="34.33203125" customWidth="1"/>
-    <col min="4" max="4" width="12.6640625" customWidth="1"/>
-    <col min="5" max="5" width="15.6640625" customWidth="1"/>
+    <col min="1" max="1" width="20.6640625" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" customWidth="1"/>
+    <col min="3" max="3" width="16.83203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="C1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="1">
+        <v>12121</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C2" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="1">
+        <v>12122</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>6</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="1">
-        <v>1</v>
-      </c>
-      <c r="B2" s="1">
-        <v>12121</v>
-      </c>
-      <c r="C2" s="1">
-        <v>12121</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="1">
-        <v>2</v>
-      </c>
-      <c r="B3" s="1">
-        <v>12122</v>
-      </c>
-      <c r="C3" s="1">
-        <v>12122</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>